<commit_message>
Commented isues are fixed
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Goutham\Desktop\gitLearn\github-practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C19E763C-A656-4EC7-AB41-627CC31A4970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88749012-8C56-4D68-A54D-660ED2971459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,32 +25,103 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
-  <si>
-    <t>dewded</t>
-  </si>
-  <si>
-    <t>wdswds</t>
-  </si>
-  <si>
-    <t>dddd</t>
-  </si>
-  <si>
-    <t>ddddd</t>
-  </si>
-  <si>
-    <t>ddd</t>
-  </si>
-  <si>
-    <t>dd</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
+  <si>
+    <t>SL</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>section</t>
+  </si>
+  <si>
+    <t>phoneno</t>
+  </si>
+  <si>
+    <t>course1</t>
+  </si>
+  <si>
+    <t>course2</t>
+  </si>
+  <si>
+    <t>course3</t>
+  </si>
+  <si>
+    <t>Bala Lakshmi</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>891852432</t>
+  </si>
+  <si>
+    <t>Kannada</t>
+  </si>
+  <si>
+    <t>Tamil</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Anudeep</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>887624262</t>
+  </si>
+  <si>
+    <t>Telugu</t>
+  </si>
+  <si>
+    <t>English</t>
+  </si>
+  <si>
+    <t>Marati</t>
+  </si>
+  <si>
+    <t>Goutham</t>
+  </si>
+  <si>
+    <t>887624261</t>
+  </si>
+  <si>
+    <t>Urdu</t>
+  </si>
+  <si>
+    <t>Rama</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>887624223</t>
+  </si>
+  <si>
+    <t>Soumya</t>
+  </si>
+  <si>
+    <t>887624211</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -66,7 +137,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -74,12 +145,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -360,62 +451,145 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:G10"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C3" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="D3" t="s">
+      <c r="B4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="E3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3">
-        <v>222</v>
+      <c r="B5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D10" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="G10" t="s">
-        <v>0</v>
+      <c r="B6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>